<commit_message>
adding multivariate weighted least squares linear regression
</commit_message>
<xml_diff>
--- a/InputData/Clean/EnvironmentalData/All-Environmental-Variables-Wide.xlsx
+++ b/InputData/Clean/EnvironmentalData/All-Environmental-Variables-Wide.xlsx
@@ -1705,6 +1705,9 @@
       <c r="I38">
         <v>-0.18</v>
       </c>
+      <c r="J38">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2">
@@ -1738,6 +1741,9 @@
       <c r="I39">
         <v>-0.175</v>
       </c>
+      <c r="J39">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2">
@@ -1771,6 +1777,9 @@
       <c r="I40">
         <v>-0.18</v>
       </c>
+      <c r="J40">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2">
@@ -1804,6 +1813,9 @@
       <c r="I41">
         <v>-0.19</v>
       </c>
+      <c r="J41">
+        <v>0.10036601</v>
+      </c>
       <c r="K41">
         <v>0</v>
       </c>
@@ -1840,6 +1852,9 @@
           <t>PBR</t>
         </is>
       </c>
+      <c r="J42">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2">
@@ -1855,6 +1870,9 @@
           <t>PBR</t>
         </is>
       </c>
+      <c r="J43">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2">
@@ -1888,6 +1906,9 @@
       <c r="I44">
         <v>-0.19</v>
       </c>
+      <c r="J44">
+        <v>0.10036601</v>
+      </c>
       <c r="K44">
         <v>0</v>
       </c>
@@ -1942,6 +1963,9 @@
       <c r="I45">
         <v>-0.14</v>
       </c>
+      <c r="J45">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2">
@@ -1975,6 +1999,9 @@
       <c r="I46">
         <v>-0.2</v>
       </c>
+      <c r="J46">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2">
@@ -2008,6 +2035,9 @@
       <c r="I47">
         <v>-0.2</v>
       </c>
+      <c r="J47">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2">
@@ -2041,6 +2071,9 @@
       <c r="I48">
         <v>-0.2</v>
       </c>
+      <c r="J48">
+        <v>0.10036601</v>
+      </c>
       <c r="K48">
         <v>0</v>
       </c>
@@ -2077,6 +2110,9 @@
           <t>PBR</t>
         </is>
       </c>
+      <c r="J49">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2">
@@ -2092,6 +2128,9 @@
           <t>PBR</t>
         </is>
       </c>
+      <c r="J50">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2">
@@ -2125,6 +2164,9 @@
       <c r="I51">
         <v>-0.19</v>
       </c>
+      <c r="J51">
+        <v>0.10036601</v>
+      </c>
       <c r="K51">
         <v>0</v>
       </c>
@@ -2179,6 +2221,9 @@
       <c r="I52">
         <v>-0.18</v>
       </c>
+      <c r="J52">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2">
@@ -2195,7 +2240,7 @@
         </is>
       </c>
       <c r="J53">
-        <v>0.1003660100008334</v>
+        <v>0.10036601</v>
       </c>
     </row>
     <row r="54">
@@ -2212,6 +2257,9 @@
           <t>PBR</t>
         </is>
       </c>
+      <c r="J54">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2">
@@ -2227,6 +2275,9 @@
           <t>PBR</t>
         </is>
       </c>
+      <c r="J55">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2">
@@ -2242,6 +2293,9 @@
           <t>PBR</t>
         </is>
       </c>
+      <c r="J56">
+        <v>0.10036601</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2">
@@ -2256,6 +2310,9 @@
         <is>
           <t>PBR</t>
         </is>
+      </c>
+      <c r="J57">
+        <v>0.10036601</v>
       </c>
     </row>
     <row r="58">

</xml_diff>

<commit_message>
added in dli control
</commit_message>
<xml_diff>
--- a/InputData/Clean/EnvironmentalData/All-Environmental-Variables-Wide.xlsx
+++ b/InputData/Clean/EnvironmentalData/All-Environmental-Variables-Wide.xlsx
@@ -6616,6 +6616,9 @@
       <c r="F191">
         <v>7.84</v>
       </c>
+      <c r="J191">
+        <v>3.4128</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2">
@@ -8755,6 +8758,9 @@
       <c r="I259">
         <v>-1.15</v>
       </c>
+      <c r="J259">
+        <v>2.9376</v>
+      </c>
       <c r="K259">
         <v>0</v>
       </c>
@@ -8959,6 +8965,9 @@
       <c r="I264">
         <v>-5.45</v>
       </c>
+      <c r="J264">
+        <v>2.8944</v>
+      </c>
       <c r="K264">
         <v>0</v>
       </c>
@@ -9163,6 +9172,9 @@
       <c r="I269">
         <v>-5.46</v>
       </c>
+      <c r="J269">
+        <v>0.864</v>
+      </c>
       <c r="K269">
         <v>1</v>
       </c>
@@ -10081,6 +10093,9 @@
       <c r="I292">
         <v>-0.62</v>
       </c>
+      <c r="J292">
+        <v>1.7712</v>
+      </c>
       <c r="K292">
         <v>0</v>
       </c>
@@ -10255,6 +10270,9 @@
       <c r="I296">
         <v>-0.63</v>
       </c>
+      <c r="J296">
+        <v>1.6848</v>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2">
@@ -10375,6 +10393,9 @@
       <c r="I299">
         <v>2.95</v>
       </c>
+      <c r="J299">
+        <v>2.7216</v>
+      </c>
       <c r="K299">
         <v>0</v>
       </c>
@@ -11332,6 +11353,9 @@
       <c r="I323">
         <v>-1.26</v>
       </c>
+      <c r="J323">
+        <v>3.024</v>
+      </c>
       <c r="K323">
         <v>9</v>
       </c>
@@ -11746,6 +11770,9 @@
       <c r="I333">
         <v>-3.255</v>
       </c>
+      <c r="J333">
+        <v>2.6784</v>
+      </c>
       <c r="K333">
         <v>0</v>
       </c>
@@ -11953,6 +11980,9 @@
       <c r="I338">
         <v>-3.26</v>
       </c>
+      <c r="J338">
+        <v>2.8512</v>
+      </c>
       <c r="K338">
         <v>0</v>
       </c>
@@ -12073,6 +12103,9 @@
       <c r="I341">
         <v>-3.17</v>
       </c>
+      <c r="J341">
+        <v>2.7216</v>
+      </c>
       <c r="K341">
         <v>0</v>
       </c>
@@ -12378,6 +12411,9 @@
       </c>
       <c r="I349">
         <v>-3.32</v>
+      </c>
+      <c r="J349">
+        <v>3.2832</v>
       </c>
       <c r="K349">
         <v>0</v>

</xml_diff>